<commit_message>
GSB f58035a9-3f48-5688-905c-fe2544edc46e A: platform archive
</commit_message>
<xml_diff>
--- a/samples/sample_impact.xlsx
+++ b/samples/sample_impact.xlsx
@@ -16,6 +16,7 @@
     <sheet name="审计示例" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="名称" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="搬移演示" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="偏离示例" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="单价">参数!$B$2</definedName>
@@ -515,6 +516,117 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>C 列为 =A{行}+$B$1 向下填充（C5 被改错）；E 列两种模板各半（平票不报）</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <f>A2+$B$1</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>A2*2</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>A2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3">
+        <f>A3+$B$1</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>A3*2</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>B1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4">
+        <f>A4+$B$1</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>A4+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5</v>
+      </c>
+      <c r="C5">
+        <f>A4+$B$1</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>A5+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6">
+        <f>A6+$B$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7">
+        <f>A7+$B$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>8</v>
+      </c>
+      <c r="C8">
+        <f>A8+$B$1</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
GSB f58035a9-3f48-5688-905c-fe2544edc46e B: platform archive
</commit_message>
<xml_diff>
--- a/samples/sample_impact.xlsx
+++ b/samples/sample_impact.xlsx
@@ -16,6 +16,7 @@
     <sheet name="审计示例" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="名称" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="搬移演示" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="同列偏离" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="单价">参数!$B$2</definedName>
@@ -515,6 +516,224 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>数量</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>单价</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" t="n">
+        <v>10</v>
+      </c>
+      <c r="C2">
+        <f>A2*$B$1</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>A2+1</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>SUM(A2:A3)</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>参数!B2</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>A2+B2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3">
+        <f>A3*$B$1</f>
+        <v/>
+      </c>
+      <c r="E3">
+        <f>A3+1</f>
+        <v/>
+      </c>
+      <c r="G3">
+        <f>SUM(A3:A4)</f>
+        <v/>
+      </c>
+      <c r="I3">
+        <f>参数!B3</f>
+        <v/>
+      </c>
+      <c r="K3">
+        <f>A3+B3</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B4" t="n">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <f>A4*$B$1</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>A4*2</f>
+        <v/>
+      </c>
+      <c r="G4">
+        <f>SUM(A4:A5)</f>
+        <v/>
+      </c>
+      <c r="I4">
+        <f>参数!B4</f>
+        <v/>
+      </c>
+      <c r="K4">
+        <f>A4+B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B5" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5">
+        <f>A5*$B$1</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>A5*2</f>
+        <v/>
+      </c>
+      <c r="I5">
+        <f>参数!$B$2</f>
+        <v/>
+      </c>
+      <c r="K5">
+        <f>A5-$B$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>6</v>
+      </c>
+      <c r="B6" t="n">
+        <v>10</v>
+      </c>
+      <c r="C6">
+        <f>A6*B6</f>
+        <v/>
+      </c>
+      <c r="I6">
+        <f>参数!B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>7</v>
+      </c>
+      <c r="B7" t="n">
+        <v>10</v>
+      </c>
+      <c r="C7">
+        <f>A7*$B$1</f>
+        <v/>
+      </c>
+      <c r="K7">
+        <f>A7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8">
+        <f>A8*$B$1</f>
+        <v/>
+      </c>
+      <c r="K8">
+        <f>Z8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>9</v>
+      </c>
+      <c r="B9" t="n">
+        <v>10</v>
+      </c>
+      <c r="C9">
+        <f>A9*$B$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B10" t="n">
+        <v>10</v>
+      </c>
+      <c r="C10">
+        <f>A10*$B$1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>11</v>
+      </c>
+      <c r="B11" t="n">
+        <v>10</v>
+      </c>
+      <c r="C11">
+        <f>A11*$B$1</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>